<commit_message>
New snapshot and sync
</commit_message>
<xml_diff>
--- a/Ps2 games.xlsx
+++ b/Ps2 games.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Collection'!$A$1:$I$213</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Collection'!$A$1:$I$216</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$B$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -141,8 +141,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CollectionTable" displayName="CollectionTable" ref="A1:I213" headerRowCount="1">
-  <autoFilter ref="A1:I213"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CollectionTable" displayName="CollectionTable" ref="A1:I216" headerRowCount="1">
+  <autoFilter ref="A1:I216"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Platform"/>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I213"/>
+  <dimension ref="A1:I216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5926,7 +5926,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Grim Fandango</t>
+          <t>Grim Fandango Remastered</t>
         </is>
       </c>
       <c r="D177" t="inlineStr"/>
@@ -5934,7 +5934,11 @@
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr"/>
-      <c r="I177" t="inlineStr"/>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>New &amp; Sealed</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -6133,7 +6137,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Made in Abyss: Binary Star Falling into Darkness</t>
+          <t>Little nightmares II</t>
         </is>
       </c>
       <c r="D186" t="inlineStr"/>
@@ -6141,11 +6145,7 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="inlineStr"/>
-      <c r="I186" t="inlineStr">
-        <is>
-          <t>Maybe switch it with the collector</t>
-        </is>
-      </c>
+      <c r="I186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Mass Effect Andromeda</t>
+          <t>Made in Abyss: Binary Star Falling into Darkness</t>
         </is>
       </c>
       <c r="D187" t="inlineStr"/>
@@ -6168,7 +6168,11 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="inlineStr"/>
-      <c r="I187" t="inlineStr"/>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Maybe switch it with the collector</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -6183,7 +6187,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>MediEvil</t>
+          <t>Mass Effect Andromeda</t>
         </is>
       </c>
       <c r="D188" t="inlineStr"/>
@@ -6206,7 +6210,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Monster Hunter: World</t>
+          <t>MediEvil</t>
         </is>
       </c>
       <c r="D189" t="inlineStr"/>
@@ -6214,11 +6218,7 @@
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="inlineStr"/>
-      <c r="I189" t="inlineStr">
-        <is>
-          <t>Disc slightly ruined, buy the boxed version</t>
-        </is>
-      </c>
+      <c r="I189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Nier: Automata The End of Yorha Edition</t>
+          <t>Monster Hunter: World</t>
         </is>
       </c>
       <c r="D190" t="inlineStr"/>
@@ -6241,7 +6241,11 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr"/>
-      <c r="I190" t="inlineStr"/>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Disc slightly ruined, buy the boxed version</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -6256,7 +6260,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Nioh</t>
+          <t>Nier: Automata The End of Yorha Edition</t>
         </is>
       </c>
       <c r="D191" t="inlineStr"/>
@@ -6279,7 +6283,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Overwatch Origins Edition</t>
+          <t>Nioh</t>
         </is>
       </c>
       <c r="D192" t="inlineStr"/>
@@ -6302,7 +6306,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Ratchet &amp; Clank</t>
+          <t>Overwatch Origins Edition</t>
         </is>
       </c>
       <c r="D193" t="inlineStr"/>
@@ -6325,7 +6329,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Red Dead Redemption II</t>
+          <t>Ratchet &amp; Clank</t>
         </is>
       </c>
       <c r="D194" t="inlineStr"/>
@@ -6348,7 +6352,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Resident Evil 2</t>
+          <t>Red Dead Redemption II</t>
         </is>
       </c>
       <c r="D195" t="inlineStr"/>
@@ -6371,7 +6375,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Resident Evil 3</t>
+          <t>Resident Evil 2</t>
         </is>
       </c>
       <c r="D196" t="inlineStr"/>
@@ -6394,7 +6398,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Resisent Evil 4</t>
+          <t>Resident Evil 3</t>
         </is>
       </c>
       <c r="D197" t="inlineStr"/>
@@ -6417,7 +6421,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Shadow of The Tomb Raider</t>
+          <t>Resisent Evil 4</t>
         </is>
       </c>
       <c r="D198" t="inlineStr"/>
@@ -6440,7 +6444,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>SWORD ART ONLINE Hollow Realization</t>
+          <t>Shadow of The Tomb Raider</t>
         </is>
       </c>
       <c r="D199" t="inlineStr"/>
@@ -6463,19 +6467,23 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Terraria</t>
+          <t>Sonic Mania</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Cartonata</t>
         </is>
       </c>
       <c r="E200" t="inlineStr"/>
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="inlineStr"/>
-      <c r="I200" t="inlineStr"/>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>The cover inside is a bit torn</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -6490,7 +6498,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>The Elder Scrolls V SKYRIM Special Edition</t>
+          <t>Stray</t>
         </is>
       </c>
       <c r="D201" t="inlineStr"/>
@@ -6498,7 +6506,11 @@
       <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="inlineStr"/>
-      <c r="I201" t="inlineStr"/>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Cartoline</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -6513,7 +6525,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>The Evil Within</t>
+          <t>SWORD ART ONLINE Hollow Realization</t>
         </is>
       </c>
       <c r="D202" t="inlineStr"/>
@@ -6536,10 +6548,14 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>The Evil Within 2</t>
-        </is>
-      </c>
-      <c r="D203" t="inlineStr"/>
+          <t>Terraria</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
       <c r="E203" t="inlineStr"/>
       <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr"/>
@@ -6559,7 +6575,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>The Last Guardian</t>
+          <t>The Elder Scrolls V SKYRIM Special Edition</t>
         </is>
       </c>
       <c r="D204" t="inlineStr"/>
@@ -6582,7 +6598,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>The Last of Us Remastered</t>
+          <t>The Evil Within</t>
         </is>
       </c>
       <c r="D205" t="inlineStr"/>
@@ -6605,7 +6621,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Tokyo Ghoul re</t>
+          <t>The Evil Within 2</t>
         </is>
       </c>
       <c r="D206" t="inlineStr"/>
@@ -6628,7 +6644,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Tokyo Ghoul: re[Call to existence]</t>
+          <t>The Last Guardian</t>
         </is>
       </c>
       <c r="D207" t="inlineStr"/>
@@ -6651,7 +6667,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Tom Clancy's Rainbow Six Siege</t>
+          <t>The Last of Us Remastered</t>
         </is>
       </c>
       <c r="D208" t="inlineStr"/>
@@ -6674,7 +6690,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Tom Clancy's The Division 2 Washington D.C Edition</t>
+          <t>Tokyo Ghoul re</t>
         </is>
       </c>
       <c r="D209" t="inlineStr"/>
@@ -6697,7 +6713,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Until Dawn</t>
+          <t>Tokyo Ghoul: re[Call to existence]</t>
         </is>
       </c>
       <c r="D210" t="inlineStr"/>
@@ -6720,7 +6736,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Watch Dogs</t>
+          <t>Tom Clancy's Rainbow Six Siege</t>
         </is>
       </c>
       <c r="D211" t="inlineStr"/>
@@ -6743,7 +6759,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Watch Dogs 2</t>
+          <t>Tom Clancy's The Division 2 Washington D.C Edition</t>
         </is>
       </c>
       <c r="D212" t="inlineStr"/>
@@ -6766,7 +6782,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Watch dogs Legion</t>
+          <t>Until Dawn</t>
         </is>
       </c>
       <c r="D213" t="inlineStr"/>
@@ -6776,10 +6792,79 @@
       <c r="H213" t="inlineStr"/>
       <c r="I213" t="inlineStr"/>
     </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>C0213</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Watch Dogs</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr"/>
+      <c r="E214" t="inlineStr"/>
+      <c r="F214" t="inlineStr"/>
+      <c r="G214" t="inlineStr"/>
+      <c r="H214" t="inlineStr"/>
+      <c r="I214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>C0214</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Watch Dogs 2</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr"/>
+      <c r="E215" t="inlineStr"/>
+      <c r="F215" t="inlineStr"/>
+      <c r="G215" t="inlineStr"/>
+      <c r="H215" t="inlineStr"/>
+      <c r="I215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>C0215</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Watch dogs Legion</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr"/>
+      <c r="E216" t="inlineStr"/>
+      <c r="F216" t="inlineStr"/>
+      <c r="G216" t="inlineStr"/>
+      <c r="H216" t="inlineStr"/>
+      <c r="I216" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I213"/>
+  <autoFilter ref="A1:I216"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B213" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B216" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PS1,PS2,PS4,DS WII"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Sync latest collection state
</commit_message>
<xml_diff>
--- a/Ps2 games.xlsx
+++ b/Ps2 games.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Collection'!$A$1:$I$216</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Collection'!$A$1:$I$235</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$B$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -141,8 +141,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CollectionTable" displayName="CollectionTable" ref="A1:I216" headerRowCount="1">
-  <autoFilter ref="A1:I216"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CollectionTable" displayName="CollectionTable" ref="A1:I235" headerRowCount="1">
+  <autoFilter ref="A1:I235"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Platform"/>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I216"/>
+  <dimension ref="A1:I235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5209,7 +5209,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Alex Kidd in Miracle World DX</t>
+          <t>Adventure Time</t>
         </is>
       </c>
       <c r="D146" t="inlineStr"/>
@@ -5232,7 +5232,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Anthem</t>
+          <t>Alex Kidd in Miracle World DX</t>
         </is>
       </c>
       <c r="D147" t="inlineStr"/>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Armored Core VI Fires of Rubicon</t>
+          <t>Anthem</t>
         </is>
       </c>
       <c r="D148" t="inlineStr"/>
@@ -5278,7 +5278,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Batman Arkham Collection</t>
+          <t>Armored Core VI Fires of Rubicon</t>
         </is>
       </c>
       <c r="D149" t="inlineStr"/>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Batman Arkham Knight</t>
+          <t>Batman Arkham Collection</t>
         </is>
       </c>
       <c r="D150" t="inlineStr"/>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Batman Return to Arkham</t>
+          <t>Batman Arkham Knight</t>
         </is>
       </c>
       <c r="D151" t="inlineStr"/>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Battlefield 4</t>
+          <t>Batman Return to Arkham</t>
         </is>
       </c>
       <c r="D152" t="inlineStr"/>
@@ -5370,7 +5370,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>BIOSHOCK The Collectioon</t>
+          <t>Battlefield 4</t>
         </is>
       </c>
       <c r="D153" t="inlineStr"/>
@@ -5393,7 +5393,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Bloodborne</t>
+          <t>BIOSHOCK The Collectioon</t>
         </is>
       </c>
       <c r="D154" t="inlineStr"/>
@@ -5416,7 +5416,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Crash Bandicoot It's About Time</t>
+          <t>Bloodborne</t>
         </is>
       </c>
       <c r="D155" t="inlineStr"/>
@@ -5439,7 +5439,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Crash N. Sane Trilogy</t>
+          <t>Crash Bandicoot It's About Time</t>
         </is>
       </c>
       <c r="D156" t="inlineStr"/>
@@ -5462,7 +5462,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Crash Team Racing: Nitro Fueled</t>
+          <t>Crash N. Sane Trilogy</t>
         </is>
       </c>
       <c r="D157" t="inlineStr"/>
@@ -5485,14 +5485,10 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Cyberpunk 2077</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>Deluxe edition</t>
-        </is>
-      </c>
+          <t>Crash Team Racing: Nitro Fueled</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr"/>
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr"/>
@@ -5512,10 +5508,14 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Dark Souls II</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr"/>
+          <t>Cyberpunk 2077</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Deluxe edition</t>
+        </is>
+      </c>
       <c r="E159" t="inlineStr"/>
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr"/>
@@ -5535,7 +5535,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Dark Souls III</t>
+          <t>Dark Souls II</t>
         </is>
       </c>
       <c r="D160" t="inlineStr"/>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Dark Souls Remastered</t>
+          <t>Dark Souls III</t>
         </is>
       </c>
       <c r="D161" t="inlineStr"/>
@@ -5581,7 +5581,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Death Stranding</t>
+          <t>Dark Souls Remastered</t>
         </is>
       </c>
       <c r="D162" t="inlineStr"/>
@@ -5604,7 +5604,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Destiny</t>
+          <t>Death Stranding</t>
         </is>
       </c>
       <c r="D163" t="inlineStr"/>
@@ -5627,7 +5627,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>DIGIMON SURVIVE</t>
+          <t>Destiny</t>
         </is>
       </c>
       <c r="D164" t="inlineStr"/>
@@ -5650,7 +5650,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>DisHonored 2</t>
+          <t>DETROIT: become human</t>
         </is>
       </c>
       <c r="D165" t="inlineStr"/>
@@ -5673,7 +5673,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>DisHonored: La morte dell'esterno</t>
+          <t>DIGIMON SURVIVE</t>
         </is>
       </c>
       <c r="D166" t="inlineStr"/>
@@ -5696,7 +5696,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>DRAGONBALL XENOVERSE 2</t>
+          <t>DisHonored 2</t>
         </is>
       </c>
       <c r="D167" t="inlineStr"/>
@@ -5719,7 +5719,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>DRIVECLUB</t>
+          <t>DisHonored: La morte dell'esterno</t>
         </is>
       </c>
       <c r="D168" t="inlineStr"/>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Farcry5</t>
+          <t>Don't Starve Mega Pack</t>
         </is>
       </c>
       <c r="D169" t="inlineStr"/>
@@ -5765,7 +5765,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Farming Simulator</t>
+          <t>Dragon Quest XI</t>
         </is>
       </c>
       <c r="D170" t="inlineStr"/>
@@ -5788,7 +5788,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>FIFA18</t>
+          <t>DRAGONBALL XENOVERSE 2</t>
         </is>
       </c>
       <c r="D171" t="inlineStr"/>
@@ -5811,7 +5811,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Final Fantasy XV Kingslaive</t>
+          <t>DRIVECLUB</t>
         </is>
       </c>
       <c r="D172" t="inlineStr"/>
@@ -5834,7 +5834,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Final Fantasz XV</t>
+          <t>Farcry5</t>
         </is>
       </c>
       <c r="D173" t="inlineStr"/>
@@ -5857,7 +5857,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>For Honor</t>
+          <t>Farming Simulator</t>
         </is>
       </c>
       <c r="D174" t="inlineStr"/>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Ghost of Tsushima</t>
+          <t>FIFA18</t>
         </is>
       </c>
       <c r="D175" t="inlineStr"/>
@@ -5903,7 +5903,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Ghostbusters Spirits Unleashed</t>
+          <t>Final Fantasy XV Kingslaive</t>
         </is>
       </c>
       <c r="D176" t="inlineStr"/>
@@ -5926,7 +5926,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Grim Fandango Remastered</t>
+          <t>Final Fantasz XV</t>
         </is>
       </c>
       <c r="D177" t="inlineStr"/>
@@ -5934,11 +5934,7 @@
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr"/>
-      <c r="I177" t="inlineStr">
-        <is>
-          <t>New &amp; Sealed</t>
-        </is>
-      </c>
+      <c r="I177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -5953,7 +5949,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Hogwarts Legacy</t>
+          <t>For Honor</t>
         </is>
       </c>
       <c r="D178" t="inlineStr"/>
@@ -5976,7 +5972,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Horizon Zero Dawn</t>
+          <t>Ghost of Tsushima</t>
         </is>
       </c>
       <c r="D179" t="inlineStr"/>
@@ -5999,7 +5995,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Immortals Fenyx Rising</t>
+          <t>Ghostbusters Spirits Unleashed</t>
         </is>
       </c>
       <c r="D180" t="inlineStr"/>
@@ -6022,7 +6018,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Judgement</t>
+          <t>Gravity rush</t>
         </is>
       </c>
       <c r="D181" t="inlineStr"/>
@@ -6045,7 +6041,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>KINGDOM HEARTS III</t>
+          <t>Grim Fandango Remastered</t>
         </is>
       </c>
       <c r="D182" t="inlineStr"/>
@@ -6053,7 +6049,11 @@
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="inlineStr"/>
-      <c r="I182" t="inlineStr"/>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>New &amp; Sealed</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -6068,7 +6068,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Lego Avengers</t>
+          <t>Hogwarts Legacy</t>
         </is>
       </c>
       <c r="D183" t="inlineStr"/>
@@ -6091,7 +6091,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Lego Worlds</t>
+          <t>Hollow Knight</t>
         </is>
       </c>
       <c r="D184" t="inlineStr"/>
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Little nightmares</t>
+          <t>Horizon Zero Dawn</t>
         </is>
       </c>
       <c r="D185" t="inlineStr"/>
@@ -6137,7 +6137,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Little nightmares II</t>
+          <t>Immortals Fenyx Rising</t>
         </is>
       </c>
       <c r="D186" t="inlineStr"/>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Made in Abyss: Binary Star Falling into Darkness</t>
+          <t>It takes two</t>
         </is>
       </c>
       <c r="D187" t="inlineStr"/>
@@ -6168,11 +6168,7 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="inlineStr"/>
-      <c r="I187" t="inlineStr">
-        <is>
-          <t>Maybe switch it with the collector</t>
-        </is>
-      </c>
+      <c r="I187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -6187,7 +6183,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Mass Effect Andromeda</t>
+          <t>Judgement</t>
         </is>
       </c>
       <c r="D188" t="inlineStr"/>
@@ -6210,7 +6206,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>MediEvil</t>
+          <t>KINGDOM HEARTS III</t>
         </is>
       </c>
       <c r="D189" t="inlineStr"/>
@@ -6233,7 +6229,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Monster Hunter: World</t>
+          <t>Lego Avengers</t>
         </is>
       </c>
       <c r="D190" t="inlineStr"/>
@@ -6241,11 +6237,7 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr"/>
-      <c r="I190" t="inlineStr">
-        <is>
-          <t>Disc slightly ruined, buy the boxed version</t>
-        </is>
-      </c>
+      <c r="I190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -6260,7 +6252,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Nier: Automata The End of Yorha Edition</t>
+          <t>Lego Worlds</t>
         </is>
       </c>
       <c r="D191" t="inlineStr"/>
@@ -6283,7 +6275,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Nioh</t>
+          <t>Little nightmares</t>
         </is>
       </c>
       <c r="D192" t="inlineStr"/>
@@ -6306,7 +6298,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Overwatch Origins Edition</t>
+          <t>Little nightmares II</t>
         </is>
       </c>
       <c r="D193" t="inlineStr"/>
@@ -6329,7 +6321,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Ratchet &amp; Clank</t>
+          <t>Little nightmares III</t>
         </is>
       </c>
       <c r="D194" t="inlineStr"/>
@@ -6352,7 +6344,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Red Dead Redemption II</t>
+          <t>Made in Abyss: Binary Star Falling into Darkness</t>
         </is>
       </c>
       <c r="D195" t="inlineStr"/>
@@ -6360,7 +6352,11 @@
       <c r="F195" t="inlineStr"/>
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="inlineStr"/>
-      <c r="I195" t="inlineStr"/>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Maybe switch it with the collector</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -6375,7 +6371,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Resident Evil 2</t>
+          <t>Mafia trilogy</t>
         </is>
       </c>
       <c r="D196" t="inlineStr"/>
@@ -6398,7 +6394,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Resident Evil 3</t>
+          <t>Mass Effect Andromeda</t>
         </is>
       </c>
       <c r="D197" t="inlineStr"/>
@@ -6421,7 +6417,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Resisent Evil 4</t>
+          <t>MediEvil</t>
         </is>
       </c>
       <c r="D198" t="inlineStr"/>
@@ -6444,7 +6440,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Shadow of The Tomb Raider</t>
+          <t>Monster Hunter: World</t>
         </is>
       </c>
       <c r="D199" t="inlineStr"/>
@@ -6452,7 +6448,11 @@
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr"/>
       <c r="H199" t="inlineStr"/>
-      <c r="I199" t="inlineStr"/>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Disc slightly ruined, buy the boxed version</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -6467,23 +6467,15 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Sonic Mania</t>
-        </is>
-      </c>
-      <c r="D200" t="inlineStr">
-        <is>
-          <t>Cartonata</t>
-        </is>
-      </c>
+          <t>Nier replicant</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr"/>
       <c r="E200" t="inlineStr"/>
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="inlineStr"/>
-      <c r="I200" t="inlineStr">
-        <is>
-          <t>The cover inside is a bit torn</t>
-        </is>
-      </c>
+      <c r="I200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -6498,7 +6490,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Stray</t>
+          <t>Nier: Automata The End of Yorha Edition</t>
         </is>
       </c>
       <c r="D201" t="inlineStr"/>
@@ -6506,11 +6498,7 @@
       <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="inlineStr"/>
-      <c r="I201" t="inlineStr">
-        <is>
-          <t>Cartoline</t>
-        </is>
-      </c>
+      <c r="I201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -6525,7 +6513,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>SWORD ART ONLINE Hollow Realization</t>
+          <t>Nioh</t>
         </is>
       </c>
       <c r="D202" t="inlineStr"/>
@@ -6548,14 +6536,10 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Terraria</t>
-        </is>
-      </c>
-      <c r="D203" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
+          <t>Okami HD</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr"/>
       <c r="E203" t="inlineStr"/>
       <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr"/>
@@ -6575,7 +6559,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>The Elder Scrolls V SKYRIM Special Edition</t>
+          <t>Outer wilds</t>
         </is>
       </c>
       <c r="D204" t="inlineStr"/>
@@ -6598,7 +6582,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>The Evil Within</t>
+          <t>Overwatch Origins Edition</t>
         </is>
       </c>
       <c r="D205" t="inlineStr"/>
@@ -6621,7 +6605,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>The Evil Within 2</t>
+          <t>Persona 5</t>
         </is>
       </c>
       <c r="D206" t="inlineStr"/>
@@ -6644,7 +6628,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>The Last Guardian</t>
+          <t>Ratchet &amp; Clank</t>
         </is>
       </c>
       <c r="D207" t="inlineStr"/>
@@ -6667,7 +6651,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>The Last of Us Remastered</t>
+          <t>Red Dead Redemption II</t>
         </is>
       </c>
       <c r="D208" t="inlineStr"/>
@@ -6690,7 +6674,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Tokyo Ghoul re</t>
+          <t>Resident Evil 2</t>
         </is>
       </c>
       <c r="D209" t="inlineStr"/>
@@ -6713,7 +6697,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Tokyo Ghoul: re[Call to existence]</t>
+          <t>Resident Evil 3</t>
         </is>
       </c>
       <c r="D210" t="inlineStr"/>
@@ -6736,7 +6720,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Tom Clancy's Rainbow Six Siege</t>
+          <t>Resident Evil Revelations</t>
         </is>
       </c>
       <c r="D211" t="inlineStr"/>
@@ -6759,7 +6743,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Tom Clancy's The Division 2 Washington D.C Edition</t>
+          <t>Resident Evil Revelations 2</t>
         </is>
       </c>
       <c r="D212" t="inlineStr"/>
@@ -6782,7 +6766,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Until Dawn</t>
+          <t>Resident Evil Village</t>
         </is>
       </c>
       <c r="D213" t="inlineStr"/>
@@ -6805,7 +6789,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Watch Dogs</t>
+          <t>Resisent Evil 4</t>
         </is>
       </c>
       <c r="D214" t="inlineStr"/>
@@ -6828,7 +6812,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Watch Dogs 2</t>
+          <t>Scribblenauts</t>
         </is>
       </c>
       <c r="D215" t="inlineStr"/>
@@ -6851,7 +6835,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Watch dogs Legion</t>
+          <t>Shadow of The Tomb Raider</t>
         </is>
       </c>
       <c r="D216" t="inlineStr"/>
@@ -6861,10 +6845,463 @@
       <c r="H216" t="inlineStr"/>
       <c r="I216" t="inlineStr"/>
     </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>C0216</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Sonic Mania</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Cartonata</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr"/>
+      <c r="F217" t="inlineStr"/>
+      <c r="G217" t="inlineStr"/>
+      <c r="H217" t="inlineStr"/>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>The cover inside is a bit torn</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>C0217</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Stray</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr"/>
+      <c r="E218" t="inlineStr"/>
+      <c r="F218" t="inlineStr"/>
+      <c r="G218" t="inlineStr"/>
+      <c r="H218" t="inlineStr"/>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Cartoline</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>C0218</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>SWORD ART ONLINE Hollow Realization</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr"/>
+      <c r="E219" t="inlineStr"/>
+      <c r="F219" t="inlineStr"/>
+      <c r="G219" t="inlineStr"/>
+      <c r="H219" t="inlineStr"/>
+      <c r="I219" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>C0219</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Terraria</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr"/>
+      <c r="F220" t="inlineStr"/>
+      <c r="G220" t="inlineStr"/>
+      <c r="H220" t="inlineStr"/>
+      <c r="I220" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>C0220</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>The Binding of Isaac: Afterbirth</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr"/>
+      <c r="E221" t="inlineStr"/>
+      <c r="F221" t="inlineStr"/>
+      <c r="G221" t="inlineStr"/>
+      <c r="H221" t="inlineStr"/>
+      <c r="I221" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>C0221</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>The Elder Scrolls V SKYRIM Special Edition</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr"/>
+      <c r="E222" t="inlineStr"/>
+      <c r="F222" t="inlineStr"/>
+      <c r="G222" t="inlineStr"/>
+      <c r="H222" t="inlineStr"/>
+      <c r="I222" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>C0222</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>The Evil Within</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr"/>
+      <c r="E223" t="inlineStr"/>
+      <c r="F223" t="inlineStr"/>
+      <c r="G223" t="inlineStr"/>
+      <c r="H223" t="inlineStr"/>
+      <c r="I223" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>C0223</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>The Evil Within 2</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr"/>
+      <c r="E224" t="inlineStr"/>
+      <c r="F224" t="inlineStr"/>
+      <c r="G224" t="inlineStr"/>
+      <c r="H224" t="inlineStr"/>
+      <c r="I224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>C0224</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>The Last Guardian</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr"/>
+      <c r="E225" t="inlineStr"/>
+      <c r="F225" t="inlineStr"/>
+      <c r="G225" t="inlineStr"/>
+      <c r="H225" t="inlineStr"/>
+      <c r="I225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>C0225</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>The Last of Us part II</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr"/>
+      <c r="E226" t="inlineStr"/>
+      <c r="F226" t="inlineStr"/>
+      <c r="G226" t="inlineStr"/>
+      <c r="H226" t="inlineStr"/>
+      <c r="I226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>C0226</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>The Last of Us Remastered</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr"/>
+      <c r="E227" t="inlineStr"/>
+      <c r="F227" t="inlineStr"/>
+      <c r="G227" t="inlineStr"/>
+      <c r="H227" t="inlineStr"/>
+      <c r="I227" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>C0227</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Tokyo Ghoul re</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr"/>
+      <c r="E228" t="inlineStr"/>
+      <c r="F228" t="inlineStr"/>
+      <c r="G228" t="inlineStr"/>
+      <c r="H228" t="inlineStr"/>
+      <c r="I228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>C0228</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Tokyo Ghoul: re[Call to existence]</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr"/>
+      <c r="E229" t="inlineStr"/>
+      <c r="F229" t="inlineStr"/>
+      <c r="G229" t="inlineStr"/>
+      <c r="H229" t="inlineStr"/>
+      <c r="I229" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>C0229</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Tom Clancy's Rainbow Six Siege</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr"/>
+      <c r="E230" t="inlineStr"/>
+      <c r="F230" t="inlineStr"/>
+      <c r="G230" t="inlineStr"/>
+      <c r="H230" t="inlineStr"/>
+      <c r="I230" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>C0230</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Tom Clancy's The Division 2 Washington D.C Edition</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr"/>
+      <c r="E231" t="inlineStr"/>
+      <c r="F231" t="inlineStr"/>
+      <c r="G231" t="inlineStr"/>
+      <c r="H231" t="inlineStr"/>
+      <c r="I231" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>C0231</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Until Dawn</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr"/>
+      <c r="E232" t="inlineStr"/>
+      <c r="F232" t="inlineStr"/>
+      <c r="G232" t="inlineStr"/>
+      <c r="H232" t="inlineStr"/>
+      <c r="I232" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>C0232</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Watch Dogs</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr"/>
+      <c r="E233" t="inlineStr"/>
+      <c r="F233" t="inlineStr"/>
+      <c r="G233" t="inlineStr"/>
+      <c r="H233" t="inlineStr"/>
+      <c r="I233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>C0233</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Watch Dogs 2</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr"/>
+      <c r="E234" t="inlineStr"/>
+      <c r="F234" t="inlineStr"/>
+      <c r="G234" t="inlineStr"/>
+      <c r="H234" t="inlineStr"/>
+      <c r="I234" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>C0234</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>PS4</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Watch dogs Legion</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr"/>
+      <c r="E235" t="inlineStr"/>
+      <c r="F235" t="inlineStr"/>
+      <c r="G235" t="inlineStr"/>
+      <c r="H235" t="inlineStr"/>
+      <c r="I235" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I216"/>
+  <autoFilter ref="A1:I235"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B216" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B235" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PS1,PS2,PS4,DS WII"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Improve collection safety and wishlist workflow
</commit_message>
<xml_diff>
--- a/Ps2 games.xlsx
+++ b/Ps2 games.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Collection'!$A$1:$I$235</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Collection'!$A$1:$K$235</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$B$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -141,9 +141,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CollectionTable" displayName="CollectionTable" ref="A1:I235" headerRowCount="1">
-  <autoFilter ref="A1:I235"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CollectionTable" displayName="CollectionTable" ref="A1:K235" headerRowCount="1">
+  <autoFilter ref="A1:K235"/>
+  <tableColumns count="11">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Platform"/>
     <tableColumn id="3" name="Title"/>
@@ -153,6 +153,8 @@
     <tableColumn id="7" name="Price"/>
     <tableColumn id="8" name="Extra"/>
     <tableColumn id="9" name="Note"/>
+    <tableColumn id="10" name="Acquired Date"/>
+    <tableColumn id="11" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -447,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I235"/>
+  <dimension ref="A1:K235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -459,6 +461,8 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,6 +509,16 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Note</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Acquired Date</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
         </is>
       </c>
     </row>
@@ -530,6 +544,8 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -553,6 +569,8 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -576,6 +594,8 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -599,6 +619,8 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -622,6 +644,8 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -645,6 +669,8 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -668,6 +694,8 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -691,6 +719,8 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -714,6 +744,8 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -737,6 +769,8 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -760,6 +794,8 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -783,6 +819,8 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -806,6 +844,8 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -829,6 +869,8 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -852,6 +894,8 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -875,6 +919,8 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -898,6 +944,8 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -921,6 +969,8 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -944,6 +994,8 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -967,6 +1019,8 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -990,6 +1044,8 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1013,6 +1069,8 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1036,6 +1094,8 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1059,6 +1119,8 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1082,6 +1144,8 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1105,6 +1169,8 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1128,6 +1194,8 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1151,6 +1219,8 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1174,6 +1244,8 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1197,6 +1269,8 @@
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1220,6 +1294,8 @@
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1243,6 +1319,8 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1266,6 +1344,8 @@
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1289,6 +1369,8 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1312,6 +1394,8 @@
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1335,6 +1419,8 @@
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1358,6 +1444,8 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1381,6 +1469,8 @@
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1404,6 +1494,8 @@
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1427,6 +1519,8 @@
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1450,6 +1544,8 @@
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1473,6 +1569,8 @@
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1496,6 +1594,8 @@
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1519,6 +1619,8 @@
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1542,6 +1644,8 @@
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1565,6 +1669,8 @@
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1588,6 +1694,8 @@
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1627,6 +1735,8 @@
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1670,6 +1780,8 @@
           <t>To sell</t>
         </is>
       </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1709,6 +1821,8 @@
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1744,6 +1858,8 @@
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1779,6 +1895,8 @@
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1814,6 +1932,8 @@
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1853,6 +1973,8 @@
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1888,6 +2010,8 @@
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1927,6 +2051,8 @@
           <t>Regenerated</t>
         </is>
       </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1966,6 +2092,8 @@
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2005,6 +2133,8 @@
           <t>Repair internal case</t>
         </is>
       </c>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2044,6 +2174,8 @@
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2083,6 +2215,8 @@
           <t>Manual and case serial don't match</t>
         </is>
       </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2118,6 +2252,8 @@
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2153,6 +2289,8 @@
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2188,6 +2326,8 @@
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2223,6 +2363,8 @@
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2262,6 +2404,8 @@
           <t>Broken case</t>
         </is>
       </c>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2297,6 +2441,8 @@
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2336,6 +2482,8 @@
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2379,6 +2527,8 @@
           <t>Regenerated</t>
         </is>
       </c>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2414,6 +2564,8 @@
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2453,6 +2605,8 @@
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2492,6 +2646,8 @@
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2531,6 +2687,8 @@
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2570,6 +2728,8 @@
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2605,6 +2765,8 @@
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2644,6 +2806,8 @@
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2683,6 +2847,8 @@
           <t>Light circular scratches</t>
         </is>
       </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2718,6 +2884,8 @@
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2761,6 +2929,8 @@
           <t>Resurface</t>
         </is>
       </c>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2800,6 +2970,8 @@
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2843,6 +3015,8 @@
           <t>Light circular scratches</t>
         </is>
       </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2878,6 +3052,8 @@
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2913,6 +3089,8 @@
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2948,6 +3126,8 @@
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr"/>
       <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2983,6 +3163,8 @@
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3022,6 +3204,8 @@
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3061,6 +3245,8 @@
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3096,6 +3282,8 @@
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3131,6 +3319,8 @@
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3174,6 +3364,8 @@
           <t>Light circular scratches</t>
         </is>
       </c>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3209,6 +3401,8 @@
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3244,6 +3438,8 @@
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr"/>
       <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3287,6 +3483,8 @@
           <t>Light circular scratches</t>
         </is>
       </c>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3322,6 +3520,8 @@
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr"/>
       <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3357,6 +3557,8 @@
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3396,6 +3598,8 @@
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3431,6 +3635,8 @@
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3470,6 +3676,8 @@
         </is>
       </c>
       <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3509,6 +3717,8 @@
         </is>
       </c>
       <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3544,6 +3754,8 @@
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3583,6 +3795,8 @@
         </is>
       </c>
       <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3622,6 +3836,8 @@
           <t>Light circular scratches</t>
         </is>
       </c>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3649,6 +3865,8 @@
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3676,6 +3894,8 @@
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr"/>
       <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3703,6 +3923,8 @@
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3742,6 +3964,8 @@
         </is>
       </c>
       <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3781,6 +4005,8 @@
           <t>Light circular scratches</t>
         </is>
       </c>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3820,6 +4046,8 @@
           <t>Circular scratches</t>
         </is>
       </c>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3847,6 +4075,8 @@
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3886,6 +4116,8 @@
           <t>Test and resurface</t>
         </is>
       </c>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3921,6 +4153,8 @@
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3960,6 +4194,8 @@
         </is>
       </c>
       <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3995,6 +4231,8 @@
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4030,6 +4268,8 @@
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -4057,6 +4297,8 @@
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4092,6 +4334,8 @@
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4131,6 +4375,8 @@
         </is>
       </c>
       <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4166,6 +4412,8 @@
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4201,6 +4449,8 @@
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4240,6 +4490,8 @@
         </is>
       </c>
       <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4283,6 +4535,8 @@
           <t>Small crack in the case</t>
         </is>
       </c>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4326,6 +4580,8 @@
           <t>Regenerated</t>
         </is>
       </c>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4365,6 +4621,8 @@
         </is>
       </c>
       <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4404,6 +4662,8 @@
         </is>
       </c>
       <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4439,6 +4699,8 @@
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4478,6 +4740,8 @@
         </is>
       </c>
       <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4513,6 +4777,8 @@
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4548,6 +4814,8 @@
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr"/>
       <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4583,6 +4851,8 @@
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4618,6 +4888,8 @@
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr"/>
       <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4653,6 +4925,8 @@
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4692,6 +4966,8 @@
         </is>
       </c>
       <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4735,6 +5011,8 @@
           <t>Test</t>
         </is>
       </c>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4770,6 +5048,8 @@
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr"/>
       <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4809,6 +5089,8 @@
         </is>
       </c>
       <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4844,6 +5126,8 @@
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="inlineStr"/>
       <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4879,6 +5163,8 @@
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4918,6 +5204,8 @@
           <t>Regenerate</t>
         </is>
       </c>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4957,6 +5245,8 @@
           <t>Regenerate</t>
         </is>
       </c>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4996,6 +5286,8 @@
         </is>
       </c>
       <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -5035,6 +5327,8 @@
           <t>Broken case</t>
         </is>
       </c>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -5074,6 +5368,8 @@
         </is>
       </c>
       <c r="I142" t="inlineStr"/>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -5117,6 +5413,8 @@
           <t>Regenerate</t>
         </is>
       </c>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -5156,6 +5454,8 @@
         </is>
       </c>
       <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -5195,6 +5495,8 @@
         </is>
       </c>
       <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -5218,6 +5520,8 @@
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr"/>
       <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -5241,6 +5545,8 @@
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr"/>
       <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -5264,6 +5570,8 @@
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr"/>
       <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -5287,6 +5595,8 @@
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr"/>
       <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5310,6 +5620,8 @@
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr"/>
       <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -5333,6 +5645,8 @@
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr"/>
       <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -5356,6 +5670,8 @@
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr"/>
       <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -5379,6 +5695,8 @@
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr"/>
       <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -5402,6 +5720,8 @@
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -5425,6 +5745,8 @@
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr"/>
       <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -5448,6 +5770,8 @@
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr"/>
       <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -5471,6 +5795,8 @@
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr"/>
       <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -5494,6 +5820,8 @@
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr"/>
       <c r="I158" t="inlineStr"/>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -5521,6 +5849,8 @@
       <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr"/>
       <c r="I159" t="inlineStr"/>
+      <c r="J159" t="inlineStr"/>
+      <c r="K159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -5544,6 +5874,8 @@
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="inlineStr"/>
       <c r="I160" t="inlineStr"/>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -5567,6 +5899,8 @@
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="inlineStr"/>
       <c r="I161" t="inlineStr"/>
+      <c r="J161" t="inlineStr"/>
+      <c r="K161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -5590,6 +5924,8 @@
       <c r="G162" t="inlineStr"/>
       <c r="H162" t="inlineStr"/>
       <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -5613,6 +5949,8 @@
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="inlineStr"/>
       <c r="I163" t="inlineStr"/>
+      <c r="J163" t="inlineStr"/>
+      <c r="K163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -5636,6 +5974,8 @@
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="inlineStr"/>
       <c r="I164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
+      <c r="K164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -5659,6 +5999,8 @@
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="inlineStr"/>
       <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
+      <c r="K165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -5682,6 +6024,8 @@
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="inlineStr"/>
       <c r="I166" t="inlineStr"/>
+      <c r="J166" t="inlineStr"/>
+      <c r="K166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -5705,6 +6049,8 @@
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="inlineStr"/>
       <c r="I167" t="inlineStr"/>
+      <c r="J167" t="inlineStr"/>
+      <c r="K167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -5728,6 +6074,8 @@
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="inlineStr"/>
       <c r="I168" t="inlineStr"/>
+      <c r="J168" t="inlineStr"/>
+      <c r="K168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -5751,6 +6099,8 @@
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr"/>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -5774,6 +6124,8 @@
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="inlineStr"/>
       <c r="I170" t="inlineStr"/>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -5797,6 +6149,8 @@
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="inlineStr"/>
       <c r="I171" t="inlineStr"/>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -5820,6 +6174,8 @@
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="inlineStr"/>
       <c r="I172" t="inlineStr"/>
+      <c r="J172" t="inlineStr"/>
+      <c r="K172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -5843,6 +6199,8 @@
       <c r="G173" t="inlineStr"/>
       <c r="H173" t="inlineStr"/>
       <c r="I173" t="inlineStr"/>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -5866,6 +6224,8 @@
       <c r="G174" t="inlineStr"/>
       <c r="H174" t="inlineStr"/>
       <c r="I174" t="inlineStr"/>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -5889,6 +6249,8 @@
       <c r="G175" t="inlineStr"/>
       <c r="H175" t="inlineStr"/>
       <c r="I175" t="inlineStr"/>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -5912,6 +6274,8 @@
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="inlineStr"/>
       <c r="I176" t="inlineStr"/>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -5935,6 +6299,8 @@
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr"/>
       <c r="I177" t="inlineStr"/>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -5958,6 +6324,8 @@
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="inlineStr"/>
       <c r="I178" t="inlineStr"/>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -5981,6 +6349,8 @@
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="inlineStr"/>
       <c r="I179" t="inlineStr"/>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -6004,6 +6374,8 @@
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="inlineStr"/>
       <c r="I180" t="inlineStr"/>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -6027,6 +6399,8 @@
       <c r="G181" t="inlineStr"/>
       <c r="H181" t="inlineStr"/>
       <c r="I181" t="inlineStr"/>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -6054,6 +6428,8 @@
           <t>New &amp; Sealed</t>
         </is>
       </c>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -6077,6 +6453,8 @@
       <c r="G183" t="inlineStr"/>
       <c r="H183" t="inlineStr"/>
       <c r="I183" t="inlineStr"/>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -6100,6 +6478,8 @@
       <c r="G184" t="inlineStr"/>
       <c r="H184" t="inlineStr"/>
       <c r="I184" t="inlineStr"/>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -6123,6 +6503,8 @@
       <c r="G185" t="inlineStr"/>
       <c r="H185" t="inlineStr"/>
       <c r="I185" t="inlineStr"/>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -6146,6 +6528,8 @@
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="inlineStr"/>
       <c r="I186" t="inlineStr"/>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -6169,6 +6553,8 @@
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="inlineStr"/>
       <c r="I187" t="inlineStr"/>
+      <c r="J187" t="inlineStr"/>
+      <c r="K187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -6192,6 +6578,8 @@
       <c r="G188" t="inlineStr"/>
       <c r="H188" t="inlineStr"/>
       <c r="I188" t="inlineStr"/>
+      <c r="J188" t="inlineStr"/>
+      <c r="K188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -6215,6 +6603,8 @@
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="inlineStr"/>
       <c r="I189" t="inlineStr"/>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -6238,6 +6628,8 @@
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr"/>
       <c r="I190" t="inlineStr"/>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -6261,6 +6653,8 @@
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="inlineStr"/>
       <c r="I191" t="inlineStr"/>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -6284,6 +6678,8 @@
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="inlineStr"/>
       <c r="I192" t="inlineStr"/>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -6307,6 +6703,8 @@
       <c r="G193" t="inlineStr"/>
       <c r="H193" t="inlineStr"/>
       <c r="I193" t="inlineStr"/>
+      <c r="J193" t="inlineStr"/>
+      <c r="K193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -6330,6 +6728,8 @@
       <c r="G194" t="inlineStr"/>
       <c r="H194" t="inlineStr"/>
       <c r="I194" t="inlineStr"/>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -6357,6 +6757,8 @@
           <t>Maybe switch it with the collector</t>
         </is>
       </c>
+      <c r="J195" t="inlineStr"/>
+      <c r="K195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -6380,6 +6782,8 @@
       <c r="G196" t="inlineStr"/>
       <c r="H196" t="inlineStr"/>
       <c r="I196" t="inlineStr"/>
+      <c r="J196" t="inlineStr"/>
+      <c r="K196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -6403,6 +6807,8 @@
       <c r="G197" t="inlineStr"/>
       <c r="H197" t="inlineStr"/>
       <c r="I197" t="inlineStr"/>
+      <c r="J197" t="inlineStr"/>
+      <c r="K197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -6426,6 +6832,8 @@
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="inlineStr"/>
       <c r="I198" t="inlineStr"/>
+      <c r="J198" t="inlineStr"/>
+      <c r="K198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -6453,6 +6861,8 @@
           <t>Disc slightly ruined, buy the boxed version</t>
         </is>
       </c>
+      <c r="J199" t="inlineStr"/>
+      <c r="K199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -6476,6 +6886,8 @@
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="inlineStr"/>
       <c r="I200" t="inlineStr"/>
+      <c r="J200" t="inlineStr"/>
+      <c r="K200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -6499,6 +6911,8 @@
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="inlineStr"/>
       <c r="I201" t="inlineStr"/>
+      <c r="J201" t="inlineStr"/>
+      <c r="K201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -6522,6 +6936,8 @@
       <c r="G202" t="inlineStr"/>
       <c r="H202" t="inlineStr"/>
       <c r="I202" t="inlineStr"/>
+      <c r="J202" t="inlineStr"/>
+      <c r="K202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -6545,6 +6961,8 @@
       <c r="G203" t="inlineStr"/>
       <c r="H203" t="inlineStr"/>
       <c r="I203" t="inlineStr"/>
+      <c r="J203" t="inlineStr"/>
+      <c r="K203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -6568,6 +6986,8 @@
       <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr"/>
       <c r="I204" t="inlineStr"/>
+      <c r="J204" t="inlineStr"/>
+      <c r="K204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -6591,6 +7011,8 @@
       <c r="G205" t="inlineStr"/>
       <c r="H205" t="inlineStr"/>
       <c r="I205" t="inlineStr"/>
+      <c r="J205" t="inlineStr"/>
+      <c r="K205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -6614,6 +7036,8 @@
       <c r="G206" t="inlineStr"/>
       <c r="H206" t="inlineStr"/>
       <c r="I206" t="inlineStr"/>
+      <c r="J206" t="inlineStr"/>
+      <c r="K206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -6637,6 +7061,8 @@
       <c r="G207" t="inlineStr"/>
       <c r="H207" t="inlineStr"/>
       <c r="I207" t="inlineStr"/>
+      <c r="J207" t="inlineStr"/>
+      <c r="K207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -6660,6 +7086,8 @@
       <c r="G208" t="inlineStr"/>
       <c r="H208" t="inlineStr"/>
       <c r="I208" t="inlineStr"/>
+      <c r="J208" t="inlineStr"/>
+      <c r="K208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -6683,6 +7111,8 @@
       <c r="G209" t="inlineStr"/>
       <c r="H209" t="inlineStr"/>
       <c r="I209" t="inlineStr"/>
+      <c r="J209" t="inlineStr"/>
+      <c r="K209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -6706,6 +7136,8 @@
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="inlineStr"/>
       <c r="I210" t="inlineStr"/>
+      <c r="J210" t="inlineStr"/>
+      <c r="K210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -6729,6 +7161,8 @@
       <c r="G211" t="inlineStr"/>
       <c r="H211" t="inlineStr"/>
       <c r="I211" t="inlineStr"/>
+      <c r="J211" t="inlineStr"/>
+      <c r="K211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -6752,6 +7186,8 @@
       <c r="G212" t="inlineStr"/>
       <c r="H212" t="inlineStr"/>
       <c r="I212" t="inlineStr"/>
+      <c r="J212" t="inlineStr"/>
+      <c r="K212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -6775,6 +7211,8 @@
       <c r="G213" t="inlineStr"/>
       <c r="H213" t="inlineStr"/>
       <c r="I213" t="inlineStr"/>
+      <c r="J213" t="inlineStr"/>
+      <c r="K213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -6798,6 +7236,8 @@
       <c r="G214" t="inlineStr"/>
       <c r="H214" t="inlineStr"/>
       <c r="I214" t="inlineStr"/>
+      <c r="J214" t="inlineStr"/>
+      <c r="K214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -6821,6 +7261,8 @@
       <c r="G215" t="inlineStr"/>
       <c r="H215" t="inlineStr"/>
       <c r="I215" t="inlineStr"/>
+      <c r="J215" t="inlineStr"/>
+      <c r="K215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -6844,6 +7286,8 @@
       <c r="G216" t="inlineStr"/>
       <c r="H216" t="inlineStr"/>
       <c r="I216" t="inlineStr"/>
+      <c r="J216" t="inlineStr"/>
+      <c r="K216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -6875,6 +7319,8 @@
           <t>The cover inside is a bit torn</t>
         </is>
       </c>
+      <c r="J217" t="inlineStr"/>
+      <c r="K217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -6902,6 +7348,8 @@
           <t>Cartoline</t>
         </is>
       </c>
+      <c r="J218" t="inlineStr"/>
+      <c r="K218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -6925,6 +7373,8 @@
       <c r="G219" t="inlineStr"/>
       <c r="H219" t="inlineStr"/>
       <c r="I219" t="inlineStr"/>
+      <c r="J219" t="inlineStr"/>
+      <c r="K219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -6952,6 +7402,8 @@
       <c r="G220" t="inlineStr"/>
       <c r="H220" t="inlineStr"/>
       <c r="I220" t="inlineStr"/>
+      <c r="J220" t="inlineStr"/>
+      <c r="K220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -6975,6 +7427,8 @@
       <c r="G221" t="inlineStr"/>
       <c r="H221" t="inlineStr"/>
       <c r="I221" t="inlineStr"/>
+      <c r="J221" t="inlineStr"/>
+      <c r="K221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -6998,6 +7452,8 @@
       <c r="G222" t="inlineStr"/>
       <c r="H222" t="inlineStr"/>
       <c r="I222" t="inlineStr"/>
+      <c r="J222" t="inlineStr"/>
+      <c r="K222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -7021,6 +7477,8 @@
       <c r="G223" t="inlineStr"/>
       <c r="H223" t="inlineStr"/>
       <c r="I223" t="inlineStr"/>
+      <c r="J223" t="inlineStr"/>
+      <c r="K223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -7044,6 +7502,8 @@
       <c r="G224" t="inlineStr"/>
       <c r="H224" t="inlineStr"/>
       <c r="I224" t="inlineStr"/>
+      <c r="J224" t="inlineStr"/>
+      <c r="K224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -7067,6 +7527,8 @@
       <c r="G225" t="inlineStr"/>
       <c r="H225" t="inlineStr"/>
       <c r="I225" t="inlineStr"/>
+      <c r="J225" t="inlineStr"/>
+      <c r="K225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -7090,6 +7552,8 @@
       <c r="G226" t="inlineStr"/>
       <c r="H226" t="inlineStr"/>
       <c r="I226" t="inlineStr"/>
+      <c r="J226" t="inlineStr"/>
+      <c r="K226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -7113,6 +7577,8 @@
       <c r="G227" t="inlineStr"/>
       <c r="H227" t="inlineStr"/>
       <c r="I227" t="inlineStr"/>
+      <c r="J227" t="inlineStr"/>
+      <c r="K227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -7136,6 +7602,8 @@
       <c r="G228" t="inlineStr"/>
       <c r="H228" t="inlineStr"/>
       <c r="I228" t="inlineStr"/>
+      <c r="J228" t="inlineStr"/>
+      <c r="K228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -7159,6 +7627,8 @@
       <c r="G229" t="inlineStr"/>
       <c r="H229" t="inlineStr"/>
       <c r="I229" t="inlineStr"/>
+      <c r="J229" t="inlineStr"/>
+      <c r="K229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -7182,6 +7652,8 @@
       <c r="G230" t="inlineStr"/>
       <c r="H230" t="inlineStr"/>
       <c r="I230" t="inlineStr"/>
+      <c r="J230" t="inlineStr"/>
+      <c r="K230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -7205,6 +7677,8 @@
       <c r="G231" t="inlineStr"/>
       <c r="H231" t="inlineStr"/>
       <c r="I231" t="inlineStr"/>
+      <c r="J231" t="inlineStr"/>
+      <c r="K231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -7228,6 +7702,8 @@
       <c r="G232" t="inlineStr"/>
       <c r="H232" t="inlineStr"/>
       <c r="I232" t="inlineStr"/>
+      <c r="J232" t="inlineStr"/>
+      <c r="K232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -7251,6 +7727,8 @@
       <c r="G233" t="inlineStr"/>
       <c r="H233" t="inlineStr"/>
       <c r="I233" t="inlineStr"/>
+      <c r="J233" t="inlineStr"/>
+      <c r="K233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -7274,6 +7752,8 @@
       <c r="G234" t="inlineStr"/>
       <c r="H234" t="inlineStr"/>
       <c r="I234" t="inlineStr"/>
+      <c r="J234" t="inlineStr"/>
+      <c r="K234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -7297,9 +7777,11 @@
       <c r="G235" t="inlineStr"/>
       <c r="H235" t="inlineStr"/>
       <c r="I235" t="inlineStr"/>
+      <c r="J235" t="inlineStr"/>
+      <c r="K235" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I235"/>
+  <autoFilter ref="A1:K235"/>
   <dataValidations count="1">
     <dataValidation sqref="B2:B235" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PS1,PS2,PS4,DS WII"</formula1>

</xml_diff>